<commit_message>
Update figure outputs and refactor script naming
Updated and renamed figure files and data outputs to align with new figure numbering (e.g., fig6 to fig5, fig5 to fig4, etc.), removed obsolete files, and adjusted script references and output paths accordingly. Refactored R scripts to match new figure structure, improved plotting logic, and updated data export locations. These changes ensure consistency between code, output files, and manuscript figure references.
</commit_message>
<xml_diff>
--- a/Outcome/Publish/figure_data/fig2.xlsx
+++ b/Outcome/Publish/figure_data/fig2.xlsx
@@ -6,14 +6,18 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="panel A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="panel C" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="panelB" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="panelC" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="panelE" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="panelF" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="460">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="474">
   <si>
     <t xml:space="preserve">Shortname</t>
   </si>
@@ -1393,6 +1397,48 @@
   </si>
   <si>
     <t xml:space="preserve">26. Chikungunya</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AgeGroup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AgeGroupID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max_tag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outcome</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Others</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5-9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20-39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40-59</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outcome_Fill</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
   </si>
 </sst>
 </file>
@@ -22850,4 +22896,4218 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>460</v>
+      </c>
+      <c r="B1" t="s">
+        <v>461</v>
+      </c>
+      <c r="C1" t="s">
+        <v>462</v>
+      </c>
+      <c r="D1" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>464</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1257443.09356982</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>464</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" t="n">
+        <v>653657.716757474</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>464</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" t="n">
+        <v>778335.599275723</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>464</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>465</v>
+      </c>
+      <c r="D5" t="n">
+        <v>410123.920688537</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>466</v>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" t="n">
+        <v>207210.406276195</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>466</v>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" t="n">
+        <v>673512.419055442</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>466</v>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" t="n">
+        <v>195085.354133745</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>466</v>
+      </c>
+      <c r="B9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" t="s">
+        <v>465</v>
+      </c>
+      <c r="D9" t="n">
+        <v>410266.63549073</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>467</v>
+      </c>
+      <c r="B10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" t="n">
+        <v>506614.23767102</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>467</v>
+      </c>
+      <c r="B11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" t="n">
+        <v>316456.043334976</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>467</v>
+      </c>
+      <c r="B12" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" t="n">
+        <v>150953.40760811</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>467</v>
+      </c>
+      <c r="B13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>465</v>
+      </c>
+      <c r="D13" t="n">
+        <v>179593.807880794</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>468</v>
+      </c>
+      <c r="B14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" t="s">
+        <v>19</v>
+      </c>
+      <c r="D14" t="n">
+        <v>247009.701346544</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>468</v>
+      </c>
+      <c r="B15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D15" t="n">
+        <v>228775.52818226</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>468</v>
+      </c>
+      <c r="B16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" t="n">
+        <v>80702.3493339277</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>468</v>
+      </c>
+      <c r="B17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" t="s">
+        <v>465</v>
+      </c>
+      <c r="D17" t="n">
+        <v>183659.029471305</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>469</v>
+      </c>
+      <c r="B18" t="n">
+        <v>5</v>
+      </c>
+      <c r="C18" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" t="n">
+        <v>291134.379172665</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>469</v>
+      </c>
+      <c r="B19" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" t="s">
+        <v>19</v>
+      </c>
+      <c r="D19" t="n">
+        <v>929183.598146722</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>469</v>
+      </c>
+      <c r="B20" t="n">
+        <v>5</v>
+      </c>
+      <c r="C20" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" t="n">
+        <v>441897.75352447</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>469</v>
+      </c>
+      <c r="B21" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" t="s">
+        <v>465</v>
+      </c>
+      <c r="D21" t="n">
+        <v>736636.991080393</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>470</v>
+      </c>
+      <c r="B22" t="n">
+        <v>6</v>
+      </c>
+      <c r="C22" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" t="n">
+        <v>627996.515626952</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>470</v>
+      </c>
+      <c r="B23" t="n">
+        <v>6</v>
+      </c>
+      <c r="C23" t="s">
+        <v>19</v>
+      </c>
+      <c r="D23" t="n">
+        <v>574225.006020735</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>470</v>
+      </c>
+      <c r="B24" t="n">
+        <v>6</v>
+      </c>
+      <c r="C24" t="s">
+        <v>16</v>
+      </c>
+      <c r="D24" t="n">
+        <v>153375.300212957</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>470</v>
+      </c>
+      <c r="B25" t="n">
+        <v>6</v>
+      </c>
+      <c r="C25" t="s">
+        <v>465</v>
+      </c>
+      <c r="D25" t="n">
+        <v>401809.73923787</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>471</v>
+      </c>
+      <c r="B26" t="n">
+        <v>7</v>
+      </c>
+      <c r="C26" t="s">
+        <v>10</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1610710.70529812</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>471</v>
+      </c>
+      <c r="B27" t="n">
+        <v>7</v>
+      </c>
+      <c r="C27" t="s">
+        <v>19</v>
+      </c>
+      <c r="D27" t="n">
+        <v>282733.321002064</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>471</v>
+      </c>
+      <c r="B28" t="n">
+        <v>7</v>
+      </c>
+      <c r="C28" t="s">
+        <v>16</v>
+      </c>
+      <c r="D28" t="n">
+        <v>48021.1745600166</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>471</v>
+      </c>
+      <c r="B29" t="n">
+        <v>7</v>
+      </c>
+      <c r="C29" t="s">
+        <v>465</v>
+      </c>
+      <c r="D29" t="n">
+        <v>182634.26604043</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>460</v>
+      </c>
+      <c r="B1" t="s">
+        <v>461</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" t="s">
+        <v>463</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>464</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>464</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>92</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>464</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>464</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>158</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>464</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>176</v>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>464</v>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>203</v>
+      </c>
+      <c r="D7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>464</v>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>237</v>
+      </c>
+      <c r="D8" t="n">
+        <v>7</v>
+      </c>
+      <c r="E8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>464</v>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>262</v>
+      </c>
+      <c r="D9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>464</v>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>291</v>
+      </c>
+      <c r="D10" t="n">
+        <v>9</v>
+      </c>
+      <c r="E10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>467</v>
+      </c>
+      <c r="B11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>467</v>
+      </c>
+      <c r="B12" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" t="s">
+        <v>92</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>467</v>
+      </c>
+      <c r="B13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>127</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" t="s">
+        <v>17</v>
+      </c>
+      <c r="G13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>467</v>
+      </c>
+      <c r="B14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" t="s">
+        <v>158</v>
+      </c>
+      <c r="D14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" t="s">
+        <v>17</v>
+      </c>
+      <c r="G14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>467</v>
+      </c>
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="s">
+        <v>176</v>
+      </c>
+      <c r="D15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" t="s">
+        <v>19</v>
+      </c>
+      <c r="F15" t="s">
+        <v>11</v>
+      </c>
+      <c r="G15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>467</v>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="s">
+        <v>203</v>
+      </c>
+      <c r="D16" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" t="s">
+        <v>19</v>
+      </c>
+      <c r="F16" t="s">
+        <v>11</v>
+      </c>
+      <c r="G16" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>467</v>
+      </c>
+      <c r="B17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>237</v>
+      </c>
+      <c r="D17" t="n">
+        <v>7</v>
+      </c>
+      <c r="E17" t="s">
+        <v>16</v>
+      </c>
+      <c r="F17" t="s">
+        <v>17</v>
+      </c>
+      <c r="G17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>467</v>
+      </c>
+      <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" t="s">
+        <v>262</v>
+      </c>
+      <c r="D18" t="n">
+        <v>8</v>
+      </c>
+      <c r="E18" t="s">
+        <v>19</v>
+      </c>
+      <c r="F18" t="s">
+        <v>11</v>
+      </c>
+      <c r="G18" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>467</v>
+      </c>
+      <c r="B19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" t="s">
+        <v>291</v>
+      </c>
+      <c r="D19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G19" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>468</v>
+      </c>
+      <c r="B20" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="s">
+        <v>16</v>
+      </c>
+      <c r="F20" t="s">
+        <v>17</v>
+      </c>
+      <c r="G20" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>468</v>
+      </c>
+      <c r="B21" t="n">
+        <v>4</v>
+      </c>
+      <c r="C21" t="s">
+        <v>92</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" t="s">
+        <v>16</v>
+      </c>
+      <c r="F21" t="s">
+        <v>17</v>
+      </c>
+      <c r="G21" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>468</v>
+      </c>
+      <c r="B22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C22" t="s">
+        <v>127</v>
+      </c>
+      <c r="D22" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" t="s">
+        <v>16</v>
+      </c>
+      <c r="F22" t="s">
+        <v>17</v>
+      </c>
+      <c r="G22" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>468</v>
+      </c>
+      <c r="B23" t="n">
+        <v>4</v>
+      </c>
+      <c r="C23" t="s">
+        <v>158</v>
+      </c>
+      <c r="D23" t="n">
+        <v>4</v>
+      </c>
+      <c r="E23" t="s">
+        <v>16</v>
+      </c>
+      <c r="F23" t="s">
+        <v>17</v>
+      </c>
+      <c r="G23" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>468</v>
+      </c>
+      <c r="B24" t="n">
+        <v>4</v>
+      </c>
+      <c r="C24" t="s">
+        <v>176</v>
+      </c>
+      <c r="D24" t="n">
+        <v>5</v>
+      </c>
+      <c r="E24" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G24" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>468</v>
+      </c>
+      <c r="B25" t="n">
+        <v>4</v>
+      </c>
+      <c r="C25" t="s">
+        <v>203</v>
+      </c>
+      <c r="D25" t="n">
+        <v>6</v>
+      </c>
+      <c r="E25" t="s">
+        <v>16</v>
+      </c>
+      <c r="F25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G25" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>468</v>
+      </c>
+      <c r="B26" t="n">
+        <v>4</v>
+      </c>
+      <c r="C26" t="s">
+        <v>237</v>
+      </c>
+      <c r="D26" t="n">
+        <v>7</v>
+      </c>
+      <c r="E26" t="s">
+        <v>16</v>
+      </c>
+      <c r="F26" t="s">
+        <v>17</v>
+      </c>
+      <c r="G26" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>468</v>
+      </c>
+      <c r="B27" t="n">
+        <v>4</v>
+      </c>
+      <c r="C27" t="s">
+        <v>262</v>
+      </c>
+      <c r="D27" t="n">
+        <v>8</v>
+      </c>
+      <c r="E27" t="s">
+        <v>19</v>
+      </c>
+      <c r="F27" t="s">
+        <v>11</v>
+      </c>
+      <c r="G27" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>468</v>
+      </c>
+      <c r="B28" t="n">
+        <v>4</v>
+      </c>
+      <c r="C28" t="s">
+        <v>291</v>
+      </c>
+      <c r="D28" t="n">
+        <v>9</v>
+      </c>
+      <c r="E28" t="s">
+        <v>19</v>
+      </c>
+      <c r="F28" t="s">
+        <v>11</v>
+      </c>
+      <c r="G28" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>469</v>
+      </c>
+      <c r="B29" t="n">
+        <v>5</v>
+      </c>
+      <c r="C29" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="s">
+        <v>16</v>
+      </c>
+      <c r="F29" t="s">
+        <v>17</v>
+      </c>
+      <c r="G29" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>469</v>
+      </c>
+      <c r="B30" t="n">
+        <v>5</v>
+      </c>
+      <c r="C30" t="s">
+        <v>92</v>
+      </c>
+      <c r="D30" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" t="s">
+        <v>16</v>
+      </c>
+      <c r="F30" t="s">
+        <v>17</v>
+      </c>
+      <c r="G30" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>469</v>
+      </c>
+      <c r="B31" t="n">
+        <v>5</v>
+      </c>
+      <c r="C31" t="s">
+        <v>127</v>
+      </c>
+      <c r="D31" t="n">
+        <v>3</v>
+      </c>
+      <c r="E31" t="s">
+        <v>16</v>
+      </c>
+      <c r="F31" t="s">
+        <v>17</v>
+      </c>
+      <c r="G31" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>469</v>
+      </c>
+      <c r="B32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C32" t="s">
+        <v>158</v>
+      </c>
+      <c r="D32" t="n">
+        <v>4</v>
+      </c>
+      <c r="E32" t="s">
+        <v>16</v>
+      </c>
+      <c r="F32" t="s">
+        <v>17</v>
+      </c>
+      <c r="G32" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>469</v>
+      </c>
+      <c r="B33" t="n">
+        <v>5</v>
+      </c>
+      <c r="C33" t="s">
+        <v>176</v>
+      </c>
+      <c r="D33" t="n">
+        <v>5</v>
+      </c>
+      <c r="E33" t="s">
+        <v>19</v>
+      </c>
+      <c r="F33" t="s">
+        <v>11</v>
+      </c>
+      <c r="G33" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>469</v>
+      </c>
+      <c r="B34" t="n">
+        <v>5</v>
+      </c>
+      <c r="C34" t="s">
+        <v>203</v>
+      </c>
+      <c r="D34" t="n">
+        <v>6</v>
+      </c>
+      <c r="E34" t="s">
+        <v>19</v>
+      </c>
+      <c r="F34" t="s">
+        <v>11</v>
+      </c>
+      <c r="G34" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>469</v>
+      </c>
+      <c r="B35" t="n">
+        <v>5</v>
+      </c>
+      <c r="C35" t="s">
+        <v>237</v>
+      </c>
+      <c r="D35" t="n">
+        <v>7</v>
+      </c>
+      <c r="E35" t="s">
+        <v>10</v>
+      </c>
+      <c r="F35" t="s">
+        <v>11</v>
+      </c>
+      <c r="G35" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>469</v>
+      </c>
+      <c r="B36" t="n">
+        <v>5</v>
+      </c>
+      <c r="C36" t="s">
+        <v>262</v>
+      </c>
+      <c r="D36" t="n">
+        <v>8</v>
+      </c>
+      <c r="E36" t="s">
+        <v>19</v>
+      </c>
+      <c r="F36" t="s">
+        <v>11</v>
+      </c>
+      <c r="G36" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>469</v>
+      </c>
+      <c r="B37" t="n">
+        <v>5</v>
+      </c>
+      <c r="C37" t="s">
+        <v>291</v>
+      </c>
+      <c r="D37" t="n">
+        <v>9</v>
+      </c>
+      <c r="E37" t="s">
+        <v>19</v>
+      </c>
+      <c r="F37" t="s">
+        <v>11</v>
+      </c>
+      <c r="G37" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>470</v>
+      </c>
+      <c r="B38" t="n">
+        <v>6</v>
+      </c>
+      <c r="C38" t="s">
+        <v>12</v>
+      </c>
+      <c r="D38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" t="s">
+        <v>10</v>
+      </c>
+      <c r="F38" t="s">
+        <v>11</v>
+      </c>
+      <c r="G38" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>470</v>
+      </c>
+      <c r="B39" t="n">
+        <v>6</v>
+      </c>
+      <c r="C39" t="s">
+        <v>92</v>
+      </c>
+      <c r="D39" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" t="s">
+        <v>10</v>
+      </c>
+      <c r="F39" t="s">
+        <v>11</v>
+      </c>
+      <c r="G39" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>470</v>
+      </c>
+      <c r="B40" t="n">
+        <v>6</v>
+      </c>
+      <c r="C40" t="s">
+        <v>127</v>
+      </c>
+      <c r="D40" t="n">
+        <v>3</v>
+      </c>
+      <c r="E40" t="s">
+        <v>10</v>
+      </c>
+      <c r="F40" t="s">
+        <v>11</v>
+      </c>
+      <c r="G40" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>470</v>
+      </c>
+      <c r="B41" t="n">
+        <v>6</v>
+      </c>
+      <c r="C41" t="s">
+        <v>158</v>
+      </c>
+      <c r="D41" t="n">
+        <v>4</v>
+      </c>
+      <c r="E41" t="s">
+        <v>10</v>
+      </c>
+      <c r="F41" t="s">
+        <v>11</v>
+      </c>
+      <c r="G41" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>470</v>
+      </c>
+      <c r="B42" t="n">
+        <v>6</v>
+      </c>
+      <c r="C42" t="s">
+        <v>176</v>
+      </c>
+      <c r="D42" t="n">
+        <v>5</v>
+      </c>
+      <c r="E42" t="s">
+        <v>10</v>
+      </c>
+      <c r="F42" t="s">
+        <v>11</v>
+      </c>
+      <c r="G42" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>470</v>
+      </c>
+      <c r="B43" t="n">
+        <v>6</v>
+      </c>
+      <c r="C43" t="s">
+        <v>203</v>
+      </c>
+      <c r="D43" t="n">
+        <v>6</v>
+      </c>
+      <c r="E43" t="s">
+        <v>10</v>
+      </c>
+      <c r="F43" t="s">
+        <v>11</v>
+      </c>
+      <c r="G43" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>470</v>
+      </c>
+      <c r="B44" t="n">
+        <v>6</v>
+      </c>
+      <c r="C44" t="s">
+        <v>237</v>
+      </c>
+      <c r="D44" t="n">
+        <v>7</v>
+      </c>
+      <c r="E44" t="s">
+        <v>10</v>
+      </c>
+      <c r="F44" t="s">
+        <v>11</v>
+      </c>
+      <c r="G44" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>470</v>
+      </c>
+      <c r="B45" t="n">
+        <v>6</v>
+      </c>
+      <c r="C45" t="s">
+        <v>262</v>
+      </c>
+      <c r="D45" t="n">
+        <v>8</v>
+      </c>
+      <c r="E45" t="s">
+        <v>10</v>
+      </c>
+      <c r="F45" t="s">
+        <v>11</v>
+      </c>
+      <c r="G45" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>470</v>
+      </c>
+      <c r="B46" t="n">
+        <v>6</v>
+      </c>
+      <c r="C46" t="s">
+        <v>291</v>
+      </c>
+      <c r="D46" t="n">
+        <v>9</v>
+      </c>
+      <c r="E46" t="s">
+        <v>19</v>
+      </c>
+      <c r="F46" t="s">
+        <v>11</v>
+      </c>
+      <c r="G46" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s">
+        <v>466</v>
+      </c>
+      <c r="B47" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" t="s">
+        <v>12</v>
+      </c>
+      <c r="D47" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>11</v>
+      </c>
+      <c r="G47" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s">
+        <v>466</v>
+      </c>
+      <c r="B48" t="n">
+        <v>2</v>
+      </c>
+      <c r="C48" t="s">
+        <v>92</v>
+      </c>
+      <c r="D48" t="n">
+        <v>2</v>
+      </c>
+      <c r="E48" t="s">
+        <v>14</v>
+      </c>
+      <c r="F48" t="s">
+        <v>11</v>
+      </c>
+      <c r="G48" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s">
+        <v>466</v>
+      </c>
+      <c r="B49" t="n">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>127</v>
+      </c>
+      <c r="D49" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" t="s">
+        <v>16</v>
+      </c>
+      <c r="F49" t="s">
+        <v>17</v>
+      </c>
+      <c r="G49" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s">
+        <v>466</v>
+      </c>
+      <c r="B50" t="n">
+        <v>2</v>
+      </c>
+      <c r="C50" t="s">
+        <v>158</v>
+      </c>
+      <c r="D50" t="n">
+        <v>4</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>11</v>
+      </c>
+      <c r="G50" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s">
+        <v>466</v>
+      </c>
+      <c r="B51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C51" t="s">
+        <v>176</v>
+      </c>
+      <c r="D51" t="n">
+        <v>5</v>
+      </c>
+      <c r="E51" t="s">
+        <v>19</v>
+      </c>
+      <c r="F51" t="s">
+        <v>11</v>
+      </c>
+      <c r="G51" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s">
+        <v>466</v>
+      </c>
+      <c r="B52" t="n">
+        <v>2</v>
+      </c>
+      <c r="C52" t="s">
+        <v>203</v>
+      </c>
+      <c r="D52" t="n">
+        <v>6</v>
+      </c>
+      <c r="E52" t="s">
+        <v>19</v>
+      </c>
+      <c r="F52" t="s">
+        <v>11</v>
+      </c>
+      <c r="G52" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s">
+        <v>466</v>
+      </c>
+      <c r="B53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" t="s">
+        <v>237</v>
+      </c>
+      <c r="D53" t="n">
+        <v>7</v>
+      </c>
+      <c r="E53" t="s">
+        <v>19</v>
+      </c>
+      <c r="F53" t="s">
+        <v>11</v>
+      </c>
+      <c r="G53" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s">
+        <v>466</v>
+      </c>
+      <c r="B54" t="n">
+        <v>2</v>
+      </c>
+      <c r="C54" t="s">
+        <v>262</v>
+      </c>
+      <c r="D54" t="n">
+        <v>8</v>
+      </c>
+      <c r="E54" t="s">
+        <v>19</v>
+      </c>
+      <c r="F54" t="s">
+        <v>11</v>
+      </c>
+      <c r="G54" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s">
+        <v>466</v>
+      </c>
+      <c r="B55" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>291</v>
+      </c>
+      <c r="D55" t="n">
+        <v>9</v>
+      </c>
+      <c r="E55" t="s">
+        <v>19</v>
+      </c>
+      <c r="F55" t="s">
+        <v>11</v>
+      </c>
+      <c r="G55" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s">
+        <v>471</v>
+      </c>
+      <c r="B56" t="n">
+        <v>7</v>
+      </c>
+      <c r="C56" t="s">
+        <v>12</v>
+      </c>
+      <c r="D56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" t="s">
+        <v>10</v>
+      </c>
+      <c r="F56" t="s">
+        <v>11</v>
+      </c>
+      <c r="G56" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s">
+        <v>471</v>
+      </c>
+      <c r="B57" t="n">
+        <v>7</v>
+      </c>
+      <c r="C57" t="s">
+        <v>92</v>
+      </c>
+      <c r="D57" t="n">
+        <v>2</v>
+      </c>
+      <c r="E57" t="s">
+        <v>10</v>
+      </c>
+      <c r="F57" t="s">
+        <v>11</v>
+      </c>
+      <c r="G57" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s">
+        <v>471</v>
+      </c>
+      <c r="B58" t="n">
+        <v>7</v>
+      </c>
+      <c r="C58" t="s">
+        <v>127</v>
+      </c>
+      <c r="D58" t="n">
+        <v>3</v>
+      </c>
+      <c r="E58" t="s">
+        <v>10</v>
+      </c>
+      <c r="F58" t="s">
+        <v>11</v>
+      </c>
+      <c r="G58" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s">
+        <v>471</v>
+      </c>
+      <c r="B59" t="n">
+        <v>7</v>
+      </c>
+      <c r="C59" t="s">
+        <v>158</v>
+      </c>
+      <c r="D59" t="n">
+        <v>4</v>
+      </c>
+      <c r="E59" t="s">
+        <v>10</v>
+      </c>
+      <c r="F59" t="s">
+        <v>11</v>
+      </c>
+      <c r="G59" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s">
+        <v>471</v>
+      </c>
+      <c r="B60" t="n">
+        <v>7</v>
+      </c>
+      <c r="C60" t="s">
+        <v>176</v>
+      </c>
+      <c r="D60" t="n">
+        <v>5</v>
+      </c>
+      <c r="E60" t="s">
+        <v>10</v>
+      </c>
+      <c r="F60" t="s">
+        <v>11</v>
+      </c>
+      <c r="G60" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s">
+        <v>471</v>
+      </c>
+      <c r="B61" t="n">
+        <v>7</v>
+      </c>
+      <c r="C61" t="s">
+        <v>203</v>
+      </c>
+      <c r="D61" t="n">
+        <v>6</v>
+      </c>
+      <c r="E61" t="s">
+        <v>10</v>
+      </c>
+      <c r="F61" t="s">
+        <v>11</v>
+      </c>
+      <c r="G61" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s">
+        <v>471</v>
+      </c>
+      <c r="B62" t="n">
+        <v>7</v>
+      </c>
+      <c r="C62" t="s">
+        <v>237</v>
+      </c>
+      <c r="D62" t="n">
+        <v>7</v>
+      </c>
+      <c r="E62" t="s">
+        <v>10</v>
+      </c>
+      <c r="F62" t="s">
+        <v>11</v>
+      </c>
+      <c r="G62" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s">
+        <v>471</v>
+      </c>
+      <c r="B63" t="n">
+        <v>7</v>
+      </c>
+      <c r="C63" t="s">
+        <v>262</v>
+      </c>
+      <c r="D63" t="n">
+        <v>8</v>
+      </c>
+      <c r="E63" t="s">
+        <v>10</v>
+      </c>
+      <c r="F63" t="s">
+        <v>11</v>
+      </c>
+      <c r="G63" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s">
+        <v>471</v>
+      </c>
+      <c r="B64" t="n">
+        <v>7</v>
+      </c>
+      <c r="C64" t="s">
+        <v>291</v>
+      </c>
+      <c r="D64" t="n">
+        <v>9</v>
+      </c>
+      <c r="E64" t="s">
+        <v>10</v>
+      </c>
+      <c r="F64" t="s">
+        <v>11</v>
+      </c>
+      <c r="G64" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s">
+        <v>473</v>
+      </c>
+      <c r="B65" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>12</v>
+      </c>
+      <c r="D65" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" t="s">
+        <v>10</v>
+      </c>
+      <c r="F65" t="s">
+        <v>11</v>
+      </c>
+      <c r="G65" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s">
+        <v>473</v>
+      </c>
+      <c r="B66" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>92</v>
+      </c>
+      <c r="D66" t="n">
+        <v>2</v>
+      </c>
+      <c r="E66" t="s">
+        <v>10</v>
+      </c>
+      <c r="F66" t="s">
+        <v>11</v>
+      </c>
+      <c r="G66" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s">
+        <v>473</v>
+      </c>
+      <c r="B67" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C67" t="s">
+        <v>127</v>
+      </c>
+      <c r="D67" t="n">
+        <v>3</v>
+      </c>
+      <c r="E67" t="s">
+        <v>10</v>
+      </c>
+      <c r="F67" t="s">
+        <v>11</v>
+      </c>
+      <c r="G67" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s">
+        <v>473</v>
+      </c>
+      <c r="B68" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>158</v>
+      </c>
+      <c r="D68" t="n">
+        <v>4</v>
+      </c>
+      <c r="E68" t="s">
+        <v>10</v>
+      </c>
+      <c r="F68" t="s">
+        <v>11</v>
+      </c>
+      <c r="G68" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s">
+        <v>473</v>
+      </c>
+      <c r="B69" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C69" t="s">
+        <v>176</v>
+      </c>
+      <c r="D69" t="n">
+        <v>5</v>
+      </c>
+      <c r="E69" t="s">
+        <v>10</v>
+      </c>
+      <c r="F69" t="s">
+        <v>11</v>
+      </c>
+      <c r="G69" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s">
+        <v>473</v>
+      </c>
+      <c r="B70" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>203</v>
+      </c>
+      <c r="D70" t="n">
+        <v>6</v>
+      </c>
+      <c r="E70" t="s">
+        <v>19</v>
+      </c>
+      <c r="F70" t="s">
+        <v>11</v>
+      </c>
+      <c r="G70" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="s">
+        <v>473</v>
+      </c>
+      <c r="B71" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C71" t="s">
+        <v>237</v>
+      </c>
+      <c r="D71" t="n">
+        <v>7</v>
+      </c>
+      <c r="E71" t="s">
+        <v>10</v>
+      </c>
+      <c r="F71" t="s">
+        <v>11</v>
+      </c>
+      <c r="G71" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s">
+        <v>473</v>
+      </c>
+      <c r="B72" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C72" t="s">
+        <v>262</v>
+      </c>
+      <c r="D72" t="n">
+        <v>8</v>
+      </c>
+      <c r="E72" t="s">
+        <v>19</v>
+      </c>
+      <c r="F72" t="s">
+        <v>11</v>
+      </c>
+      <c r="G72" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s">
+        <v>473</v>
+      </c>
+      <c r="B73" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C73" t="s">
+        <v>291</v>
+      </c>
+      <c r="D73" t="n">
+        <v>9</v>
+      </c>
+      <c r="E73" t="s">
+        <v>19</v>
+      </c>
+      <c r="F73" t="s">
+        <v>11</v>
+      </c>
+      <c r="G73" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>460</v>
+      </c>
+      <c r="B1" t="s">
+        <v>461</v>
+      </c>
+      <c r="C1" t="s">
+        <v>462</v>
+      </c>
+      <c r="D1" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>464</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="n">
+        <v>336.080851276617</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>464</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" t="n">
+        <v>40.4357357286305</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>464</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="n">
+        <v>169.699817591538</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>464</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>465</v>
+      </c>
+      <c r="D5" t="n">
+        <v>191.654561429724</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>466</v>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" t="n">
+        <v>123.433050356455</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>466</v>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" t="n">
+        <v>35.5613447848116</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>466</v>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" t="n">
+        <v>202.728745098835</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>466</v>
+      </c>
+      <c r="B9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" t="s">
+        <v>465</v>
+      </c>
+      <c r="D9" t="n">
+        <v>75.0283032288795</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>467</v>
+      </c>
+      <c r="B10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" t="n">
+        <v>80.9761478966684</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>467</v>
+      </c>
+      <c r="B11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" t="n">
+        <v>28.3782590097662</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>467</v>
+      </c>
+      <c r="B12" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" t="n">
+        <v>205.745763807094</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>467</v>
+      </c>
+      <c r="B13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>465</v>
+      </c>
+      <c r="D13" t="n">
+        <v>70.03391855809</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>468</v>
+      </c>
+      <c r="B14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" t="n">
+        <v>66.3469031230314</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>468</v>
+      </c>
+      <c r="B15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" t="n">
+        <v>27.5016333122411</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>468</v>
+      </c>
+      <c r="B16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" t="n">
+        <v>181.560075908497</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>468</v>
+      </c>
+      <c r="B17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" t="s">
+        <v>465</v>
+      </c>
+      <c r="D17" t="n">
+        <v>67.4717672663374</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>469</v>
+      </c>
+      <c r="B18" t="n">
+        <v>5</v>
+      </c>
+      <c r="C18" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" t="n">
+        <v>638.968665995045</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>469</v>
+      </c>
+      <c r="B19" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" t="n">
+        <v>463.168177197315</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>469</v>
+      </c>
+      <c r="B20" t="n">
+        <v>5</v>
+      </c>
+      <c r="C20" t="s">
+        <v>39</v>
+      </c>
+      <c r="D20" t="n">
+        <v>211.095224336815</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>469</v>
+      </c>
+      <c r="B21" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" t="s">
+        <v>465</v>
+      </c>
+      <c r="D21" t="n">
+        <v>519.652686835759</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>470</v>
+      </c>
+      <c r="B22" t="n">
+        <v>6</v>
+      </c>
+      <c r="C22" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" t="n">
+        <v>2446.43752319239</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>470</v>
+      </c>
+      <c r="B23" t="n">
+        <v>6</v>
+      </c>
+      <c r="C23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D23" t="n">
+        <v>384.713255981969</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>470</v>
+      </c>
+      <c r="B24" t="n">
+        <v>6</v>
+      </c>
+      <c r="C24" t="s">
+        <v>54</v>
+      </c>
+      <c r="D24" t="n">
+        <v>505.262578811219</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>470</v>
+      </c>
+      <c r="B25" t="n">
+        <v>6</v>
+      </c>
+      <c r="C25" t="s">
+        <v>465</v>
+      </c>
+      <c r="D25" t="n">
+        <v>729.342289003483</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>471</v>
+      </c>
+      <c r="B26" t="n">
+        <v>7</v>
+      </c>
+      <c r="C26" t="s">
+        <v>10</v>
+      </c>
+      <c r="D26" t="n">
+        <v>8580.75685815979</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>471</v>
+      </c>
+      <c r="B27" t="n">
+        <v>7</v>
+      </c>
+      <c r="C27" t="s">
+        <v>19</v>
+      </c>
+      <c r="D27" t="n">
+        <v>269.151549583756</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>471</v>
+      </c>
+      <c r="B28" t="n">
+        <v>7</v>
+      </c>
+      <c r="C28" t="s">
+        <v>54</v>
+      </c>
+      <c r="D28" t="n">
+        <v>391.243936788619</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>471</v>
+      </c>
+      <c r="B29" t="n">
+        <v>7</v>
+      </c>
+      <c r="C29" t="s">
+        <v>465</v>
+      </c>
+      <c r="D29" t="n">
+        <v>629.570375736621</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>460</v>
+      </c>
+      <c r="B1" t="s">
+        <v>461</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" t="s">
+        <v>463</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>464</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>464</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>92</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>464</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>464</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>158</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>464</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>176</v>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>464</v>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>203</v>
+      </c>
+      <c r="D7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>464</v>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>237</v>
+      </c>
+      <c r="D8" t="n">
+        <v>7</v>
+      </c>
+      <c r="E8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>464</v>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>262</v>
+      </c>
+      <c r="D9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>464</v>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>291</v>
+      </c>
+      <c r="D10" t="n">
+        <v>9</v>
+      </c>
+      <c r="E10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>467</v>
+      </c>
+      <c r="B11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>467</v>
+      </c>
+      <c r="B12" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" t="s">
+        <v>92</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>467</v>
+      </c>
+      <c r="B13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>127</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" t="s">
+        <v>17</v>
+      </c>
+      <c r="G13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>467</v>
+      </c>
+      <c r="B14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" t="s">
+        <v>158</v>
+      </c>
+      <c r="D14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" t="s">
+        <v>17</v>
+      </c>
+      <c r="G14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>467</v>
+      </c>
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="s">
+        <v>176</v>
+      </c>
+      <c r="D15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" t="s">
+        <v>16</v>
+      </c>
+      <c r="F15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>467</v>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="s">
+        <v>203</v>
+      </c>
+      <c r="D16" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" t="s">
+        <v>17</v>
+      </c>
+      <c r="G16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>467</v>
+      </c>
+      <c r="B17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>237</v>
+      </c>
+      <c r="D17" t="n">
+        <v>7</v>
+      </c>
+      <c r="E17" t="s">
+        <v>16</v>
+      </c>
+      <c r="F17" t="s">
+        <v>17</v>
+      </c>
+      <c r="G17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>467</v>
+      </c>
+      <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" t="s">
+        <v>262</v>
+      </c>
+      <c r="D18" t="n">
+        <v>8</v>
+      </c>
+      <c r="E18" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>467</v>
+      </c>
+      <c r="B19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" t="s">
+        <v>291</v>
+      </c>
+      <c r="D19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E19" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" t="s">
+        <v>17</v>
+      </c>
+      <c r="G19" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>468</v>
+      </c>
+      <c r="B20" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="s">
+        <v>16</v>
+      </c>
+      <c r="F20" t="s">
+        <v>17</v>
+      </c>
+      <c r="G20" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>468</v>
+      </c>
+      <c r="B21" t="n">
+        <v>4</v>
+      </c>
+      <c r="C21" t="s">
+        <v>92</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" t="s">
+        <v>16</v>
+      </c>
+      <c r="F21" t="s">
+        <v>17</v>
+      </c>
+      <c r="G21" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>468</v>
+      </c>
+      <c r="B22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C22" t="s">
+        <v>127</v>
+      </c>
+      <c r="D22" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" t="s">
+        <v>16</v>
+      </c>
+      <c r="F22" t="s">
+        <v>17</v>
+      </c>
+      <c r="G22" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>468</v>
+      </c>
+      <c r="B23" t="n">
+        <v>4</v>
+      </c>
+      <c r="C23" t="s">
+        <v>158</v>
+      </c>
+      <c r="D23" t="n">
+        <v>4</v>
+      </c>
+      <c r="E23" t="s">
+        <v>16</v>
+      </c>
+      <c r="F23" t="s">
+        <v>17</v>
+      </c>
+      <c r="G23" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>468</v>
+      </c>
+      <c r="B24" t="n">
+        <v>4</v>
+      </c>
+      <c r="C24" t="s">
+        <v>176</v>
+      </c>
+      <c r="D24" t="n">
+        <v>5</v>
+      </c>
+      <c r="E24" t="s">
+        <v>16</v>
+      </c>
+      <c r="F24" t="s">
+        <v>17</v>
+      </c>
+      <c r="G24" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>468</v>
+      </c>
+      <c r="B25" t="n">
+        <v>4</v>
+      </c>
+      <c r="C25" t="s">
+        <v>203</v>
+      </c>
+      <c r="D25" t="n">
+        <v>6</v>
+      </c>
+      <c r="E25" t="s">
+        <v>16</v>
+      </c>
+      <c r="F25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G25" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>468</v>
+      </c>
+      <c r="B26" t="n">
+        <v>4</v>
+      </c>
+      <c r="C26" t="s">
+        <v>237</v>
+      </c>
+      <c r="D26" t="n">
+        <v>7</v>
+      </c>
+      <c r="E26" t="s">
+        <v>16</v>
+      </c>
+      <c r="F26" t="s">
+        <v>17</v>
+      </c>
+      <c r="G26" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>468</v>
+      </c>
+      <c r="B27" t="n">
+        <v>4</v>
+      </c>
+      <c r="C27" t="s">
+        <v>262</v>
+      </c>
+      <c r="D27" t="n">
+        <v>8</v>
+      </c>
+      <c r="E27" t="s">
+        <v>16</v>
+      </c>
+      <c r="F27" t="s">
+        <v>17</v>
+      </c>
+      <c r="G27" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>468</v>
+      </c>
+      <c r="B28" t="n">
+        <v>4</v>
+      </c>
+      <c r="C28" t="s">
+        <v>291</v>
+      </c>
+      <c r="D28" t="n">
+        <v>9</v>
+      </c>
+      <c r="E28" t="s">
+        <v>16</v>
+      </c>
+      <c r="F28" t="s">
+        <v>17</v>
+      </c>
+      <c r="G28" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>469</v>
+      </c>
+      <c r="B29" t="n">
+        <v>5</v>
+      </c>
+      <c r="C29" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="s">
+        <v>10</v>
+      </c>
+      <c r="F29" t="s">
+        <v>11</v>
+      </c>
+      <c r="G29" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>469</v>
+      </c>
+      <c r="B30" t="n">
+        <v>5</v>
+      </c>
+      <c r="C30" t="s">
+        <v>92</v>
+      </c>
+      <c r="D30" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" t="s">
+        <v>10</v>
+      </c>
+      <c r="F30" t="s">
+        <v>11</v>
+      </c>
+      <c r="G30" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>469</v>
+      </c>
+      <c r="B31" t="n">
+        <v>5</v>
+      </c>
+      <c r="C31" t="s">
+        <v>127</v>
+      </c>
+      <c r="D31" t="n">
+        <v>3</v>
+      </c>
+      <c r="E31" t="s">
+        <v>10</v>
+      </c>
+      <c r="F31" t="s">
+        <v>11</v>
+      </c>
+      <c r="G31" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>469</v>
+      </c>
+      <c r="B32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C32" t="s">
+        <v>158</v>
+      </c>
+      <c r="D32" t="n">
+        <v>4</v>
+      </c>
+      <c r="E32" t="s">
+        <v>10</v>
+      </c>
+      <c r="F32" t="s">
+        <v>11</v>
+      </c>
+      <c r="G32" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>469</v>
+      </c>
+      <c r="B33" t="n">
+        <v>5</v>
+      </c>
+      <c r="C33" t="s">
+        <v>176</v>
+      </c>
+      <c r="D33" t="n">
+        <v>5</v>
+      </c>
+      <c r="E33" t="s">
+        <v>16</v>
+      </c>
+      <c r="F33" t="s">
+        <v>17</v>
+      </c>
+      <c r="G33" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>469</v>
+      </c>
+      <c r="B34" t="n">
+        <v>5</v>
+      </c>
+      <c r="C34" t="s">
+        <v>203</v>
+      </c>
+      <c r="D34" t="n">
+        <v>6</v>
+      </c>
+      <c r="E34" t="s">
+        <v>16</v>
+      </c>
+      <c r="F34" t="s">
+        <v>17</v>
+      </c>
+      <c r="G34" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>469</v>
+      </c>
+      <c r="B35" t="n">
+        <v>5</v>
+      </c>
+      <c r="C35" t="s">
+        <v>237</v>
+      </c>
+      <c r="D35" t="n">
+        <v>7</v>
+      </c>
+      <c r="E35" t="s">
+        <v>10</v>
+      </c>
+      <c r="F35" t="s">
+        <v>11</v>
+      </c>
+      <c r="G35" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>469</v>
+      </c>
+      <c r="B36" t="n">
+        <v>5</v>
+      </c>
+      <c r="C36" t="s">
+        <v>262</v>
+      </c>
+      <c r="D36" t="n">
+        <v>8</v>
+      </c>
+      <c r="E36" t="s">
+        <v>16</v>
+      </c>
+      <c r="F36" t="s">
+        <v>17</v>
+      </c>
+      <c r="G36" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>469</v>
+      </c>
+      <c r="B37" t="n">
+        <v>5</v>
+      </c>
+      <c r="C37" t="s">
+        <v>291</v>
+      </c>
+      <c r="D37" t="n">
+        <v>9</v>
+      </c>
+      <c r="E37" t="s">
+        <v>10</v>
+      </c>
+      <c r="F37" t="s">
+        <v>11</v>
+      </c>
+      <c r="G37" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>470</v>
+      </c>
+      <c r="B38" t="n">
+        <v>6</v>
+      </c>
+      <c r="C38" t="s">
+        <v>12</v>
+      </c>
+      <c r="D38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" t="s">
+        <v>10</v>
+      </c>
+      <c r="F38" t="s">
+        <v>11</v>
+      </c>
+      <c r="G38" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>470</v>
+      </c>
+      <c r="B39" t="n">
+        <v>6</v>
+      </c>
+      <c r="C39" t="s">
+        <v>92</v>
+      </c>
+      <c r="D39" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" t="s">
+        <v>10</v>
+      </c>
+      <c r="F39" t="s">
+        <v>11</v>
+      </c>
+      <c r="G39" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>470</v>
+      </c>
+      <c r="B40" t="n">
+        <v>6</v>
+      </c>
+      <c r="C40" t="s">
+        <v>127</v>
+      </c>
+      <c r="D40" t="n">
+        <v>3</v>
+      </c>
+      <c r="E40" t="s">
+        <v>10</v>
+      </c>
+      <c r="F40" t="s">
+        <v>11</v>
+      </c>
+      <c r="G40" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>470</v>
+      </c>
+      <c r="B41" t="n">
+        <v>6</v>
+      </c>
+      <c r="C41" t="s">
+        <v>158</v>
+      </c>
+      <c r="D41" t="n">
+        <v>4</v>
+      </c>
+      <c r="E41" t="s">
+        <v>10</v>
+      </c>
+      <c r="F41" t="s">
+        <v>11</v>
+      </c>
+      <c r="G41" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>470</v>
+      </c>
+      <c r="B42" t="n">
+        <v>6</v>
+      </c>
+      <c r="C42" t="s">
+        <v>176</v>
+      </c>
+      <c r="D42" t="n">
+        <v>5</v>
+      </c>
+      <c r="E42" t="s">
+        <v>10</v>
+      </c>
+      <c r="F42" t="s">
+        <v>11</v>
+      </c>
+      <c r="G42" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>470</v>
+      </c>
+      <c r="B43" t="n">
+        <v>6</v>
+      </c>
+      <c r="C43" t="s">
+        <v>203</v>
+      </c>
+      <c r="D43" t="n">
+        <v>6</v>
+      </c>
+      <c r="E43" t="s">
+        <v>10</v>
+      </c>
+      <c r="F43" t="s">
+        <v>11</v>
+      </c>
+      <c r="G43" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>470</v>
+      </c>
+      <c r="B44" t="n">
+        <v>6</v>
+      </c>
+      <c r="C44" t="s">
+        <v>237</v>
+      </c>
+      <c r="D44" t="n">
+        <v>7</v>
+      </c>
+      <c r="E44" t="s">
+        <v>10</v>
+      </c>
+      <c r="F44" t="s">
+        <v>11</v>
+      </c>
+      <c r="G44" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>470</v>
+      </c>
+      <c r="B45" t="n">
+        <v>6</v>
+      </c>
+      <c r="C45" t="s">
+        <v>262</v>
+      </c>
+      <c r="D45" t="n">
+        <v>8</v>
+      </c>
+      <c r="E45" t="s">
+        <v>10</v>
+      </c>
+      <c r="F45" t="s">
+        <v>11</v>
+      </c>
+      <c r="G45" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>470</v>
+      </c>
+      <c r="B46" t="n">
+        <v>6</v>
+      </c>
+      <c r="C46" t="s">
+        <v>291</v>
+      </c>
+      <c r="D46" t="n">
+        <v>9</v>
+      </c>
+      <c r="E46" t="s">
+        <v>10</v>
+      </c>
+      <c r="F46" t="s">
+        <v>11</v>
+      </c>
+      <c r="G46" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s">
+        <v>466</v>
+      </c>
+      <c r="B47" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" t="s">
+        <v>12</v>
+      </c>
+      <c r="D47" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" t="s">
+        <v>10</v>
+      </c>
+      <c r="F47" t="s">
+        <v>11</v>
+      </c>
+      <c r="G47" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s">
+        <v>466</v>
+      </c>
+      <c r="B48" t="n">
+        <v>2</v>
+      </c>
+      <c r="C48" t="s">
+        <v>92</v>
+      </c>
+      <c r="D48" t="n">
+        <v>2</v>
+      </c>
+      <c r="E48" t="s">
+        <v>16</v>
+      </c>
+      <c r="F48" t="s">
+        <v>17</v>
+      </c>
+      <c r="G48" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s">
+        <v>466</v>
+      </c>
+      <c r="B49" t="n">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>127</v>
+      </c>
+      <c r="D49" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" t="s">
+        <v>16</v>
+      </c>
+      <c r="F49" t="s">
+        <v>17</v>
+      </c>
+      <c r="G49" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s">
+        <v>466</v>
+      </c>
+      <c r="B50" t="n">
+        <v>2</v>
+      </c>
+      <c r="C50" t="s">
+        <v>158</v>
+      </c>
+      <c r="D50" t="n">
+        <v>4</v>
+      </c>
+      <c r="E50" t="s">
+        <v>16</v>
+      </c>
+      <c r="F50" t="s">
+        <v>17</v>
+      </c>
+      <c r="G50" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s">
+        <v>466</v>
+      </c>
+      <c r="B51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C51" t="s">
+        <v>176</v>
+      </c>
+      <c r="D51" t="n">
+        <v>5</v>
+      </c>
+      <c r="E51" t="s">
+        <v>16</v>
+      </c>
+      <c r="F51" t="s">
+        <v>17</v>
+      </c>
+      <c r="G51" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s">
+        <v>466</v>
+      </c>
+      <c r="B52" t="n">
+        <v>2</v>
+      </c>
+      <c r="C52" t="s">
+        <v>203</v>
+      </c>
+      <c r="D52" t="n">
+        <v>6</v>
+      </c>
+      <c r="E52" t="s">
+        <v>16</v>
+      </c>
+      <c r="F52" t="s">
+        <v>17</v>
+      </c>
+      <c r="G52" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s">
+        <v>466</v>
+      </c>
+      <c r="B53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" t="s">
+        <v>237</v>
+      </c>
+      <c r="D53" t="n">
+        <v>7</v>
+      </c>
+      <c r="E53" t="s">
+        <v>16</v>
+      </c>
+      <c r="F53" t="s">
+        <v>17</v>
+      </c>
+      <c r="G53" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s">
+        <v>466</v>
+      </c>
+      <c r="B54" t="n">
+        <v>2</v>
+      </c>
+      <c r="C54" t="s">
+        <v>262</v>
+      </c>
+      <c r="D54" t="n">
+        <v>8</v>
+      </c>
+      <c r="E54" t="s">
+        <v>16</v>
+      </c>
+      <c r="F54" t="s">
+        <v>17</v>
+      </c>
+      <c r="G54" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s">
+        <v>466</v>
+      </c>
+      <c r="B55" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>291</v>
+      </c>
+      <c r="D55" t="n">
+        <v>9</v>
+      </c>
+      <c r="E55" t="s">
+        <v>16</v>
+      </c>
+      <c r="F55" t="s">
+        <v>17</v>
+      </c>
+      <c r="G55" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s">
+        <v>471</v>
+      </c>
+      <c r="B56" t="n">
+        <v>7</v>
+      </c>
+      <c r="C56" t="s">
+        <v>12</v>
+      </c>
+      <c r="D56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" t="s">
+        <v>10</v>
+      </c>
+      <c r="F56" t="s">
+        <v>11</v>
+      </c>
+      <c r="G56" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s">
+        <v>471</v>
+      </c>
+      <c r="B57" t="n">
+        <v>7</v>
+      </c>
+      <c r="C57" t="s">
+        <v>92</v>
+      </c>
+      <c r="D57" t="n">
+        <v>2</v>
+      </c>
+      <c r="E57" t="s">
+        <v>10</v>
+      </c>
+      <c r="F57" t="s">
+        <v>11</v>
+      </c>
+      <c r="G57" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s">
+        <v>471</v>
+      </c>
+      <c r="B58" t="n">
+        <v>7</v>
+      </c>
+      <c r="C58" t="s">
+        <v>127</v>
+      </c>
+      <c r="D58" t="n">
+        <v>3</v>
+      </c>
+      <c r="E58" t="s">
+        <v>10</v>
+      </c>
+      <c r="F58" t="s">
+        <v>11</v>
+      </c>
+      <c r="G58" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s">
+        <v>471</v>
+      </c>
+      <c r="B59" t="n">
+        <v>7</v>
+      </c>
+      <c r="C59" t="s">
+        <v>158</v>
+      </c>
+      <c r="D59" t="n">
+        <v>4</v>
+      </c>
+      <c r="E59" t="s">
+        <v>10</v>
+      </c>
+      <c r="F59" t="s">
+        <v>11</v>
+      </c>
+      <c r="G59" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s">
+        <v>471</v>
+      </c>
+      <c r="B60" t="n">
+        <v>7</v>
+      </c>
+      <c r="C60" t="s">
+        <v>176</v>
+      </c>
+      <c r="D60" t="n">
+        <v>5</v>
+      </c>
+      <c r="E60" t="s">
+        <v>10</v>
+      </c>
+      <c r="F60" t="s">
+        <v>11</v>
+      </c>
+      <c r="G60" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s">
+        <v>471</v>
+      </c>
+      <c r="B61" t="n">
+        <v>7</v>
+      </c>
+      <c r="C61" t="s">
+        <v>203</v>
+      </c>
+      <c r="D61" t="n">
+        <v>6</v>
+      </c>
+      <c r="E61" t="s">
+        <v>10</v>
+      </c>
+      <c r="F61" t="s">
+        <v>11</v>
+      </c>
+      <c r="G61" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s">
+        <v>471</v>
+      </c>
+      <c r="B62" t="n">
+        <v>7</v>
+      </c>
+      <c r="C62" t="s">
+        <v>237</v>
+      </c>
+      <c r="D62" t="n">
+        <v>7</v>
+      </c>
+      <c r="E62" t="s">
+        <v>10</v>
+      </c>
+      <c r="F62" t="s">
+        <v>11</v>
+      </c>
+      <c r="G62" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s">
+        <v>471</v>
+      </c>
+      <c r="B63" t="n">
+        <v>7</v>
+      </c>
+      <c r="C63" t="s">
+        <v>262</v>
+      </c>
+      <c r="D63" t="n">
+        <v>8</v>
+      </c>
+      <c r="E63" t="s">
+        <v>10</v>
+      </c>
+      <c r="F63" t="s">
+        <v>11</v>
+      </c>
+      <c r="G63" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s">
+        <v>471</v>
+      </c>
+      <c r="B64" t="n">
+        <v>7</v>
+      </c>
+      <c r="C64" t="s">
+        <v>291</v>
+      </c>
+      <c r="D64" t="n">
+        <v>9</v>
+      </c>
+      <c r="E64" t="s">
+        <v>10</v>
+      </c>
+      <c r="F64" t="s">
+        <v>11</v>
+      </c>
+      <c r="G64" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s">
+        <v>473</v>
+      </c>
+      <c r="B65" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>12</v>
+      </c>
+      <c r="D65" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" t="s">
+        <v>10</v>
+      </c>
+      <c r="F65" t="s">
+        <v>11</v>
+      </c>
+      <c r="G65" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s">
+        <v>473</v>
+      </c>
+      <c r="B66" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>92</v>
+      </c>
+      <c r="D66" t="n">
+        <v>2</v>
+      </c>
+      <c r="E66" t="s">
+        <v>10</v>
+      </c>
+      <c r="F66" t="s">
+        <v>11</v>
+      </c>
+      <c r="G66" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s">
+        <v>473</v>
+      </c>
+      <c r="B67" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C67" t="s">
+        <v>127</v>
+      </c>
+      <c r="D67" t="n">
+        <v>3</v>
+      </c>
+      <c r="E67" t="s">
+        <v>10</v>
+      </c>
+      <c r="F67" t="s">
+        <v>11</v>
+      </c>
+      <c r="G67" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s">
+        <v>473</v>
+      </c>
+      <c r="B68" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>158</v>
+      </c>
+      <c r="D68" t="n">
+        <v>4</v>
+      </c>
+      <c r="E68" t="s">
+        <v>10</v>
+      </c>
+      <c r="F68" t="s">
+        <v>11</v>
+      </c>
+      <c r="G68" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s">
+        <v>473</v>
+      </c>
+      <c r="B69" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C69" t="s">
+        <v>176</v>
+      </c>
+      <c r="D69" t="n">
+        <v>5</v>
+      </c>
+      <c r="E69" t="s">
+        <v>10</v>
+      </c>
+      <c r="F69" t="s">
+        <v>11</v>
+      </c>
+      <c r="G69" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s">
+        <v>473</v>
+      </c>
+      <c r="B70" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>203</v>
+      </c>
+      <c r="D70" t="n">
+        <v>6</v>
+      </c>
+      <c r="E70" t="s">
+        <v>10</v>
+      </c>
+      <c r="F70" t="s">
+        <v>11</v>
+      </c>
+      <c r="G70" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="s">
+        <v>473</v>
+      </c>
+      <c r="B71" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C71" t="s">
+        <v>237</v>
+      </c>
+      <c r="D71" t="n">
+        <v>7</v>
+      </c>
+      <c r="E71" t="s">
+        <v>10</v>
+      </c>
+      <c r="F71" t="s">
+        <v>11</v>
+      </c>
+      <c r="G71" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s">
+        <v>473</v>
+      </c>
+      <c r="B72" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C72" t="s">
+        <v>262</v>
+      </c>
+      <c r="D72" t="n">
+        <v>8</v>
+      </c>
+      <c r="E72" t="s">
+        <v>10</v>
+      </c>
+      <c r="F72" t="s">
+        <v>11</v>
+      </c>
+      <c r="G72" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s">
+        <v>473</v>
+      </c>
+      <c r="B73" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C73" t="s">
+        <v>291</v>
+      </c>
+      <c r="D73" t="n">
+        <v>9</v>
+      </c>
+      <c r="E73" t="s">
+        <v>10</v>
+      </c>
+      <c r="F73" t="s">
+        <v>11</v>
+      </c>
+      <c r="G73" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add suppression analysis script and update figures
Added ScriptAnalysis/7_a_suppression.R for suppression and rebound analysis, generating new data and updated visualizations for fig5. Updated and regenerated related figure files (fig2, fig5, and associated data), added fig5_a_data.csv, and updated figure_data/fig2.xlsx and fig5.xlsx. Renamed and refactored 7_a_impact_factor.R to 8_a_recovery.R, removing duplicated suppression/rebound analysis and focusing on recovery dynamics. Updated RData files to reflect new analyses.
</commit_message>
<xml_diff>
--- a/Outcome/Publish/figure_data/fig2.xlsx
+++ b/Outcome/Publish/figure_data/fig2.xlsx
@@ -22910,7 +22910,7 @@
         <v>10</v>
       </c>
       <c r="D2" t="n">
-        <v>1122035.09356982</v>
+        <v>1352767.09356982</v>
       </c>
     </row>
     <row r="3">
@@ -22924,7 +22924,7 @@
         <v>19</v>
       </c>
       <c r="D3" t="n">
-        <v>424390.716757474</v>
+        <v>668844.716757474</v>
       </c>
     </row>
     <row r="4">
@@ -22938,7 +22938,7 @@
         <v>27</v>
       </c>
       <c r="D4" t="n">
-        <v>635915.599275723</v>
+        <v>780643.599275723</v>
       </c>
     </row>
     <row r="5">
@@ -22952,7 +22952,7 @@
         <v>459</v>
       </c>
       <c r="D5" t="n">
-        <v>372089.920688537</v>
+        <v>410364.920688537</v>
       </c>
     </row>
     <row r="6">
@@ -22963,10 +22963,10 @@
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="D6" t="n">
-        <v>342927.419055442</v>
+        <v>209882.406276195</v>
       </c>
     </row>
     <row r="7">
@@ -22977,10 +22977,10 @@
         <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D7" t="n">
-        <v>177939.354133745</v>
+        <v>698234.419055442</v>
       </c>
     </row>
     <row r="8">
@@ -22991,10 +22991,10 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D8" t="n">
-        <v>177032.729009513</v>
+        <v>196487.354133745</v>
       </c>
     </row>
     <row r="9">
@@ -23008,7 +23008,7 @@
         <v>459</v>
       </c>
       <c r="D9" t="n">
-        <v>299117.312757412</v>
+        <v>411701.63549073</v>
       </c>
     </row>
     <row r="10">
@@ -23022,7 +23022,7 @@
         <v>19</v>
       </c>
       <c r="D10" t="n">
-        <v>274748.23767102</v>
+        <v>526505.23767102</v>
       </c>
     </row>
     <row r="11">
@@ -23036,7 +23036,7 @@
         <v>16</v>
       </c>
       <c r="D11" t="n">
-        <v>295964.043334976</v>
+        <v>324080.043334976</v>
       </c>
     </row>
     <row r="12">
@@ -23050,7 +23050,7 @@
         <v>14</v>
       </c>
       <c r="D12" t="n">
-        <v>137663.40760811</v>
+        <v>151456.40760811</v>
       </c>
     </row>
     <row r="13">
@@ -23064,7 +23064,7 @@
         <v>459</v>
       </c>
       <c r="D13" t="n">
-        <v>141464.807880794</v>
+        <v>181103.807880794</v>
       </c>
     </row>
     <row r="14">
@@ -23078,7 +23078,7 @@
         <v>19</v>
       </c>
       <c r="D14" t="n">
-        <v>134604.701346544</v>
+        <v>256606.701346544</v>
       </c>
     </row>
     <row r="15">
@@ -23092,7 +23092,7 @@
         <v>16</v>
       </c>
       <c r="D15" t="n">
-        <v>208241.52818226</v>
+        <v>229081.52818226</v>
       </c>
     </row>
     <row r="16">
@@ -23106,7 +23106,7 @@
         <v>14</v>
       </c>
       <c r="D16" t="n">
-        <v>73372.3493339277</v>
+        <v>81020.3493339277</v>
       </c>
     </row>
     <row r="17">
@@ -23120,7 +23120,7 @@
         <v>459</v>
       </c>
       <c r="D17" t="n">
-        <v>146601.029471305</v>
+        <v>184956.029471305</v>
       </c>
     </row>
     <row r="18">
@@ -23134,7 +23134,7 @@
         <v>10</v>
       </c>
       <c r="D18" t="n">
-        <v>223030.379172665</v>
+        <v>292727.379172665</v>
       </c>
     </row>
     <row r="19">
@@ -23148,7 +23148,7 @@
         <v>19</v>
       </c>
       <c r="D19" t="n">
-        <v>500926.598146722</v>
+        <v>960694.598146722</v>
       </c>
     </row>
     <row r="20">
@@ -23162,7 +23162,7 @@
         <v>16</v>
       </c>
       <c r="D20" t="n">
-        <v>390503.75352447</v>
+        <v>443001.75352447</v>
       </c>
     </row>
     <row r="21">
@@ -23176,7 +23176,7 @@
         <v>459</v>
       </c>
       <c r="D21" t="n">
-        <v>612843.991080393</v>
+        <v>740759.991080393</v>
       </c>
     </row>
     <row r="22">
@@ -23190,7 +23190,7 @@
         <v>10</v>
       </c>
       <c r="D22" t="n">
-        <v>493463.515626952</v>
+        <v>632294.515626952</v>
       </c>
     </row>
     <row r="23">
@@ -23204,7 +23204,7 @@
         <v>19</v>
       </c>
       <c r="D23" t="n">
-        <v>306849.006020735</v>
+        <v>589344.006020735</v>
       </c>
     </row>
     <row r="24">
@@ -23218,7 +23218,7 @@
         <v>16</v>
       </c>
       <c r="D24" t="n">
-        <v>133103.300212957</v>
+        <v>157078.300212957</v>
       </c>
     </row>
     <row r="25">
@@ -23232,7 +23232,7 @@
         <v>459</v>
       </c>
       <c r="D25" t="n">
-        <v>335025.73923787</v>
+        <v>402068.73923787</v>
       </c>
     </row>
     <row r="26">
@@ -23246,7 +23246,7 @@
         <v>10</v>
       </c>
       <c r="D26" t="n">
-        <v>1256320.70529812</v>
+        <v>1624393.70529812</v>
       </c>
     </row>
     <row r="27">
@@ -23260,7 +23260,7 @@
         <v>19</v>
       </c>
       <c r="D27" t="n">
-        <v>149106.321002064</v>
+        <v>290810.321002064</v>
       </c>
     </row>
     <row r="28">
@@ -23274,7 +23274,7 @@
         <v>16</v>
       </c>
       <c r="D28" t="n">
-        <v>39708.1745600166</v>
+        <v>50650.1745600166</v>
       </c>
     </row>
     <row r="29">
@@ -23288,7 +23288,7 @@
         <v>459</v>
       </c>
       <c r="D29" t="n">
-        <v>142650.26604043</v>
+        <v>182005.26604043</v>
       </c>
     </row>
   </sheetData>
@@ -23511,25 +23511,25 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>12</v>
+        <v>291</v>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E10" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F10" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G10" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11">
@@ -23540,10 +23540,10 @@
         <v>3</v>
       </c>
       <c r="C11" t="s">
-        <v>92</v>
+        <v>12</v>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11" t="s">
         <v>16</v>
@@ -23563,10 +23563,10 @@
         <v>3</v>
       </c>
       <c r="C12" t="s">
-        <v>127</v>
+        <v>92</v>
       </c>
       <c r="D12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E12" t="s">
         <v>16</v>
@@ -23586,10 +23586,10 @@
         <v>3</v>
       </c>
       <c r="C13" t="s">
-        <v>158</v>
+        <v>127</v>
       </c>
       <c r="D13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E13" t="s">
         <v>16</v>
@@ -23609,19 +23609,19 @@
         <v>3</v>
       </c>
       <c r="C14" t="s">
-        <v>176</v>
+        <v>158</v>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E14" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F14" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G14" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15">
@@ -23632,10 +23632,10 @@
         <v>3</v>
       </c>
       <c r="C15" t="s">
-        <v>203</v>
+        <v>176</v>
       </c>
       <c r="D15" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E15" t="s">
         <v>19</v>
@@ -23655,19 +23655,19 @@
         <v>3</v>
       </c>
       <c r="C16" t="s">
-        <v>237</v>
+        <v>203</v>
       </c>
       <c r="D16" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E16" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F16" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G16" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17">
@@ -23678,65 +23678,65 @@
         <v>3</v>
       </c>
       <c r="C17" t="s">
-        <v>262</v>
+        <v>237</v>
       </c>
       <c r="D17" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E17" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F17" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G17" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C18" t="s">
-        <v>12</v>
+        <v>262</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E18" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F18" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G18" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C19" t="s">
-        <v>92</v>
+        <v>291</v>
       </c>
       <c r="D19" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E19" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F19" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G19" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20">
@@ -23747,10 +23747,10 @@
         <v>4</v>
       </c>
       <c r="C20" t="s">
-        <v>127</v>
+        <v>12</v>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E20" t="s">
         <v>16</v>
@@ -23770,10 +23770,10 @@
         <v>4</v>
       </c>
       <c r="C21" t="s">
-        <v>158</v>
+        <v>92</v>
       </c>
       <c r="D21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E21" t="s">
         <v>16</v>
@@ -23793,19 +23793,19 @@
         <v>4</v>
       </c>
       <c r="C22" t="s">
-        <v>176</v>
+        <v>127</v>
       </c>
       <c r="D22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E22" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F22" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G22" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23">
@@ -23816,10 +23816,10 @@
         <v>4</v>
       </c>
       <c r="C23" t="s">
-        <v>203</v>
+        <v>158</v>
       </c>
       <c r="D23" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E23" t="s">
         <v>16</v>
@@ -23839,19 +23839,19 @@
         <v>4</v>
       </c>
       <c r="C24" t="s">
-        <v>237</v>
+        <v>176</v>
       </c>
       <c r="D24" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E24" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F24" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G24" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="25">
@@ -23862,33 +23862,33 @@
         <v>4</v>
       </c>
       <c r="C25" t="s">
-        <v>262</v>
+        <v>203</v>
       </c>
       <c r="D25" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E25" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F25" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G25" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C26" t="s">
-        <v>12</v>
+        <v>237</v>
       </c>
       <c r="D26" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E26" t="s">
         <v>16</v>
@@ -23902,48 +23902,48 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C27" t="s">
-        <v>92</v>
+        <v>262</v>
       </c>
       <c r="D27" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E27" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F27" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G27" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B28" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C28" t="s">
-        <v>127</v>
+        <v>291</v>
       </c>
       <c r="D28" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E28" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F28" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G28" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="29">
@@ -23954,10 +23954,10 @@
         <v>5</v>
       </c>
       <c r="C29" t="s">
-        <v>158</v>
+        <v>12</v>
       </c>
       <c r="D29" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E29" t="s">
         <v>16</v>
@@ -23977,19 +23977,19 @@
         <v>5</v>
       </c>
       <c r="C30" t="s">
-        <v>176</v>
+        <v>92</v>
       </c>
       <c r="D30" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E30" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F30" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G30" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="31">
@@ -24000,19 +24000,19 @@
         <v>5</v>
       </c>
       <c r="C31" t="s">
-        <v>203</v>
+        <v>127</v>
       </c>
       <c r="D31" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E31" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F31" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G31" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="32">
@@ -24023,19 +24023,19 @@
         <v>5</v>
       </c>
       <c r="C32" t="s">
-        <v>237</v>
+        <v>158</v>
       </c>
       <c r="D32" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E32" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F32" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G32" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="33">
@@ -24046,10 +24046,10 @@
         <v>5</v>
       </c>
       <c r="C33" t="s">
-        <v>262</v>
+        <v>176</v>
       </c>
       <c r="D33" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E33" t="s">
         <v>19</v>
@@ -24063,39 +24063,39 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B34" t="n">
+        <v>5</v>
+      </c>
+      <c r="C34" t="s">
+        <v>203</v>
+      </c>
+      <c r="D34" t="n">
         <v>6</v>
       </c>
-      <c r="C34" t="s">
-        <v>12</v>
-      </c>
-      <c r="D34" t="n">
-        <v>1</v>
-      </c>
       <c r="E34" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F34" t="s">
         <v>11</v>
       </c>
       <c r="G34" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B35" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C35" t="s">
-        <v>92</v>
+        <v>237</v>
       </c>
       <c r="D35" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E35" t="s">
         <v>10</v>
@@ -24109,48 +24109,48 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B36" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C36" t="s">
-        <v>127</v>
+        <v>262</v>
       </c>
       <c r="D36" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E36" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F36" t="s">
         <v>11</v>
       </c>
       <c r="G36" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B37" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C37" t="s">
-        <v>158</v>
+        <v>291</v>
       </c>
       <c r="D37" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E37" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F37" t="s">
         <v>11</v>
       </c>
       <c r="G37" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="38">
@@ -24161,10 +24161,10 @@
         <v>6</v>
       </c>
       <c r="C38" t="s">
-        <v>176</v>
+        <v>12</v>
       </c>
       <c r="D38" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E38" t="s">
         <v>10</v>
@@ -24184,10 +24184,10 @@
         <v>6</v>
       </c>
       <c r="C39" t="s">
-        <v>203</v>
+        <v>92</v>
       </c>
       <c r="D39" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E39" t="s">
         <v>10</v>
@@ -24207,10 +24207,10 @@
         <v>6</v>
       </c>
       <c r="C40" t="s">
-        <v>237</v>
+        <v>127</v>
       </c>
       <c r="D40" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E40" t="s">
         <v>10</v>
@@ -24230,10 +24230,10 @@
         <v>6</v>
       </c>
       <c r="C41" t="s">
-        <v>262</v>
+        <v>158</v>
       </c>
       <c r="D41" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E41" t="s">
         <v>10</v>
@@ -24247,108 +24247,108 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="B42" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C42" t="s">
-        <v>12</v>
+        <v>176</v>
       </c>
       <c r="D42" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E42" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F42" t="s">
         <v>11</v>
       </c>
       <c r="G42" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="B43" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C43" t="s">
-        <v>92</v>
+        <v>203</v>
       </c>
       <c r="D43" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E43" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F43" t="s">
         <v>11</v>
       </c>
       <c r="G43" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="B44" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C44" t="s">
-        <v>127</v>
+        <v>237</v>
       </c>
       <c r="D44" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E44" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F44" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G44" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="B45" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C45" t="s">
-        <v>158</v>
+        <v>262</v>
       </c>
       <c r="D45" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E45" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F45" t="s">
         <v>11</v>
       </c>
       <c r="G45" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="B46" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C46" t="s">
-        <v>176</v>
+        <v>291</v>
       </c>
       <c r="D46" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E46" t="s">
         <v>19</v>
@@ -24368,19 +24368,19 @@
         <v>2</v>
       </c>
       <c r="C47" t="s">
-        <v>203</v>
+        <v>12</v>
       </c>
       <c r="D47" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E47" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F47" t="s">
         <v>11</v>
       </c>
       <c r="G47" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="48">
@@ -24391,19 +24391,19 @@
         <v>2</v>
       </c>
       <c r="C48" t="s">
-        <v>237</v>
+        <v>92</v>
       </c>
       <c r="D48" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E48" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F48" t="s">
         <v>11</v>
       </c>
       <c r="G48" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="49">
@@ -24414,157 +24414,157 @@
         <v>2</v>
       </c>
       <c r="C49" t="s">
-        <v>262</v>
+        <v>127</v>
       </c>
       <c r="D49" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E49" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F49" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G49" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="B50" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C50" t="s">
-        <v>12</v>
+        <v>158</v>
       </c>
       <c r="D50" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E50" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F50" t="s">
         <v>11</v>
       </c>
       <c r="G50" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="B51" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C51" t="s">
-        <v>92</v>
+        <v>176</v>
       </c>
       <c r="D51" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E51" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F51" t="s">
         <v>11</v>
       </c>
       <c r="G51" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="B52" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C52" t="s">
-        <v>127</v>
+        <v>203</v>
       </c>
       <c r="D52" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E52" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F52" t="s">
         <v>11</v>
       </c>
       <c r="G52" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="B53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" t="s">
+        <v>237</v>
+      </c>
+      <c r="D53" t="n">
         <v>7</v>
       </c>
-      <c r="C53" t="s">
-        <v>158</v>
-      </c>
-      <c r="D53" t="n">
-        <v>4</v>
-      </c>
       <c r="E53" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F53" t="s">
         <v>11</v>
       </c>
       <c r="G53" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="B54" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C54" t="s">
-        <v>176</v>
+        <v>262</v>
       </c>
       <c r="D54" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E54" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F54" t="s">
         <v>11</v>
       </c>
       <c r="G54" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="B55" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C55" t="s">
-        <v>203</v>
+        <v>291</v>
       </c>
       <c r="D55" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E55" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F55" t="s">
         <v>11</v>
       </c>
       <c r="G55" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="56">
@@ -24575,10 +24575,10 @@
         <v>7</v>
       </c>
       <c r="C56" t="s">
-        <v>237</v>
+        <v>12</v>
       </c>
       <c r="D56" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E56" t="s">
         <v>10</v>
@@ -24598,10 +24598,10 @@
         <v>7</v>
       </c>
       <c r="C57" t="s">
-        <v>262</v>
+        <v>92</v>
       </c>
       <c r="D57" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E57" t="s">
         <v>10</v>
@@ -24615,16 +24615,16 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="B58" t="n">
-        <v>8.2</v>
+        <v>7</v>
       </c>
       <c r="C58" t="s">
-        <v>12</v>
+        <v>127</v>
       </c>
       <c r="D58" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E58" t="s">
         <v>10</v>
@@ -24638,16 +24638,16 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="B59" t="n">
-        <v>8.2</v>
+        <v>7</v>
       </c>
       <c r="C59" t="s">
-        <v>92</v>
+        <v>158</v>
       </c>
       <c r="D59" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E59" t="s">
         <v>10</v>
@@ -24661,16 +24661,16 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="B60" t="n">
-        <v>8.2</v>
+        <v>7</v>
       </c>
       <c r="C60" t="s">
-        <v>127</v>
+        <v>176</v>
       </c>
       <c r="D60" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E60" t="s">
         <v>10</v>
@@ -24684,16 +24684,16 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="B61" t="n">
-        <v>8.2</v>
+        <v>7</v>
       </c>
       <c r="C61" t="s">
-        <v>158</v>
+        <v>203</v>
       </c>
       <c r="D61" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E61" t="s">
         <v>10</v>
@@ -24707,16 +24707,16 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="B62" t="n">
-        <v>8.2</v>
+        <v>7</v>
       </c>
       <c r="C62" t="s">
-        <v>176</v>
+        <v>237</v>
       </c>
       <c r="D62" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E62" t="s">
         <v>10</v>
@@ -24730,39 +24730,39 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="B63" t="n">
-        <v>8.2</v>
+        <v>7</v>
       </c>
       <c r="C63" t="s">
-        <v>203</v>
+        <v>262</v>
       </c>
       <c r="D63" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E63" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F63" t="s">
         <v>11</v>
       </c>
       <c r="G63" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="B64" t="n">
-        <v>8.2</v>
+        <v>7</v>
       </c>
       <c r="C64" t="s">
-        <v>237</v>
+        <v>291</v>
       </c>
       <c r="D64" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E64" t="s">
         <v>10</v>
@@ -24782,18 +24782,202 @@
         <v>8.2</v>
       </c>
       <c r="C65" t="s">
+        <v>12</v>
+      </c>
+      <c r="D65" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" t="s">
+        <v>10</v>
+      </c>
+      <c r="F65" t="s">
+        <v>11</v>
+      </c>
+      <c r="G65" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s">
+        <v>467</v>
+      </c>
+      <c r="B66" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>92</v>
+      </c>
+      <c r="D66" t="n">
+        <v>2</v>
+      </c>
+      <c r="E66" t="s">
+        <v>10</v>
+      </c>
+      <c r="F66" t="s">
+        <v>11</v>
+      </c>
+      <c r="G66" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s">
+        <v>467</v>
+      </c>
+      <c r="B67" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C67" t="s">
+        <v>127</v>
+      </c>
+      <c r="D67" t="n">
+        <v>3</v>
+      </c>
+      <c r="E67" t="s">
+        <v>10</v>
+      </c>
+      <c r="F67" t="s">
+        <v>11</v>
+      </c>
+      <c r="G67" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s">
+        <v>467</v>
+      </c>
+      <c r="B68" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>158</v>
+      </c>
+      <c r="D68" t="n">
+        <v>4</v>
+      </c>
+      <c r="E68" t="s">
+        <v>10</v>
+      </c>
+      <c r="F68" t="s">
+        <v>11</v>
+      </c>
+      <c r="G68" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s">
+        <v>467</v>
+      </c>
+      <c r="B69" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C69" t="s">
+        <v>176</v>
+      </c>
+      <c r="D69" t="n">
+        <v>5</v>
+      </c>
+      <c r="E69" t="s">
+        <v>10</v>
+      </c>
+      <c r="F69" t="s">
+        <v>11</v>
+      </c>
+      <c r="G69" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s">
+        <v>467</v>
+      </c>
+      <c r="B70" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>203</v>
+      </c>
+      <c r="D70" t="n">
+        <v>6</v>
+      </c>
+      <c r="E70" t="s">
+        <v>19</v>
+      </c>
+      <c r="F70" t="s">
+        <v>11</v>
+      </c>
+      <c r="G70" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="s">
+        <v>467</v>
+      </c>
+      <c r="B71" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C71" t="s">
+        <v>237</v>
+      </c>
+      <c r="D71" t="n">
+        <v>7</v>
+      </c>
+      <c r="E71" t="s">
+        <v>10</v>
+      </c>
+      <c r="F71" t="s">
+        <v>11</v>
+      </c>
+      <c r="G71" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s">
+        <v>467</v>
+      </c>
+      <c r="B72" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C72" t="s">
         <v>262</v>
       </c>
-      <c r="D65" t="n">
+      <c r="D72" t="n">
         <v>8</v>
       </c>
-      <c r="E65" t="s">
+      <c r="E72" t="s">
         <v>19</v>
       </c>
-      <c r="F65" t="s">
-        <v>11</v>
-      </c>
-      <c r="G65" t="s">
+      <c r="F72" t="s">
+        <v>11</v>
+      </c>
+      <c r="G72" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s">
+        <v>467</v>
+      </c>
+      <c r="B73" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C73" t="s">
+        <v>291</v>
+      </c>
+      <c r="D73" t="n">
+        <v>9</v>
+      </c>
+      <c r="E73" t="s">
+        <v>19</v>
+      </c>
+      <c r="F73" t="s">
+        <v>11</v>
+      </c>
+      <c r="G73" t="s">
         <v>19</v>
       </c>
     </row>
@@ -24833,7 +25017,7 @@
         <v>10</v>
       </c>
       <c r="D2" t="n">
-        <v>318.080851276617</v>
+        <v>336.080851276617</v>
       </c>
     </row>
     <row r="3">
@@ -24844,10 +25028,10 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D3" t="n">
-        <v>161.699817591538</v>
+        <v>40.4357357286305</v>
       </c>
     </row>
     <row r="4">
@@ -24858,10 +25042,10 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>86</v>
+        <v>16</v>
       </c>
       <c r="D4" t="n">
-        <v>38</v>
+        <v>169.699817591538</v>
       </c>
     </row>
     <row r="5">
@@ -24875,7 +25059,7 @@
         <v>459</v>
       </c>
       <c r="D5" t="n">
-        <v>158.090297158354</v>
+        <v>191.654561429724</v>
       </c>
     </row>
     <row r="6">
@@ -24889,7 +25073,7 @@
         <v>10</v>
       </c>
       <c r="D6" t="n">
-        <v>117.433050356455</v>
+        <v>123.433050356455</v>
       </c>
     </row>
     <row r="7">
@@ -24903,7 +25087,7 @@
         <v>19</v>
       </c>
       <c r="D7" t="n">
-        <v>25.5613447848116</v>
+        <v>35.5613447848116</v>
       </c>
     </row>
     <row r="8">
@@ -24917,7 +25101,7 @@
         <v>16</v>
       </c>
       <c r="D8" t="n">
-        <v>187.728745098835</v>
+        <v>202.728745098835</v>
       </c>
     </row>
     <row r="9">
@@ -24931,7 +25115,7 @@
         <v>459</v>
       </c>
       <c r="D9" t="n">
-        <v>68.0283032288795</v>
+        <v>75.0283032288795</v>
       </c>
     </row>
     <row r="10">
@@ -24945,7 +25129,7 @@
         <v>10</v>
       </c>
       <c r="D10" t="n">
-        <v>69.9761478966684</v>
+        <v>81.9761478966684</v>
       </c>
     </row>
     <row r="11">
@@ -24959,7 +25143,7 @@
         <v>19</v>
       </c>
       <c r="D11" t="n">
-        <v>23.3782590097662</v>
+        <v>28.3782590097662</v>
       </c>
     </row>
     <row r="12">
@@ -24973,7 +25157,7 @@
         <v>16</v>
       </c>
       <c r="D12" t="n">
-        <v>192.745763807094</v>
+        <v>206.745763807094</v>
       </c>
     </row>
     <row r="13">
@@ -24987,7 +25171,7 @@
         <v>459</v>
       </c>
       <c r="D13" t="n">
-        <v>65.03391855809</v>
+        <v>71.03391855809</v>
       </c>
     </row>
     <row r="14">
@@ -25001,7 +25185,7 @@
         <v>10</v>
       </c>
       <c r="D14" t="n">
-        <v>63.3469031230314</v>
+        <v>66.3469031230314</v>
       </c>
     </row>
     <row r="15">
@@ -25015,7 +25199,7 @@
         <v>19</v>
       </c>
       <c r="D15" t="n">
-        <v>25.5016333122411</v>
+        <v>27.5016333122411</v>
       </c>
     </row>
     <row r="16">
@@ -25029,7 +25213,7 @@
         <v>16</v>
       </c>
       <c r="D16" t="n">
-        <v>172.560075908497</v>
+        <v>181.560075908497</v>
       </c>
     </row>
     <row r="17">
@@ -25043,7 +25227,7 @@
         <v>459</v>
       </c>
       <c r="D17" t="n">
-        <v>64.4717672663374</v>
+        <v>67.4717672663374</v>
       </c>
     </row>
     <row r="18">
@@ -25057,7 +25241,7 @@
         <v>10</v>
       </c>
       <c r="D18" t="n">
-        <v>584.968665995045</v>
+        <v>642.968665995045</v>
       </c>
     </row>
     <row r="19">
@@ -25071,7 +25255,7 @@
         <v>16</v>
       </c>
       <c r="D19" t="n">
-        <v>423.168177197315</v>
+        <v>463.168177197315</v>
       </c>
     </row>
     <row r="20">
@@ -25085,7 +25269,7 @@
         <v>39</v>
       </c>
       <c r="D20" t="n">
-        <v>191.095224336815</v>
+        <v>212.095224336815</v>
       </c>
     </row>
     <row r="21">
@@ -25099,7 +25283,7 @@
         <v>459</v>
       </c>
       <c r="D21" t="n">
-        <v>450.652686835759</v>
+        <v>519.652686835759</v>
       </c>
     </row>
     <row r="22">
@@ -25113,7 +25297,7 @@
         <v>10</v>
       </c>
       <c r="D22" t="n">
-        <v>2154.43752319239</v>
+        <v>2457.43752319239</v>
       </c>
     </row>
     <row r="23">
@@ -25127,7 +25311,7 @@
         <v>39</v>
       </c>
       <c r="D23" t="n">
-        <v>304.713255981969</v>
+        <v>386.713255981969</v>
       </c>
     </row>
     <row r="24">
@@ -25141,7 +25325,7 @@
         <v>54</v>
       </c>
       <c r="D24" t="n">
-        <v>358.262578811219</v>
+        <v>512.262578811219</v>
       </c>
     </row>
     <row r="25">
@@ -25155,7 +25339,7 @@
         <v>459</v>
       </c>
       <c r="D25" t="n">
-        <v>611.342289003483</v>
+        <v>733.342289003483</v>
       </c>
     </row>
     <row r="26">
@@ -25169,7 +25353,7 @@
         <v>10</v>
       </c>
       <c r="D26" t="n">
-        <v>7406.75685815979</v>
+        <v>8634.75685815979</v>
       </c>
     </row>
     <row r="27">
@@ -25183,7 +25367,7 @@
         <v>19</v>
       </c>
       <c r="D27" t="n">
-        <v>191.151549583756</v>
+        <v>279.151549583756</v>
       </c>
     </row>
     <row r="28">
@@ -25197,7 +25381,7 @@
         <v>54</v>
       </c>
       <c r="D28" t="n">
-        <v>258.243936788619</v>
+        <v>396.243936788619</v>
       </c>
     </row>
     <row r="29">
@@ -25211,7 +25395,7 @@
         <v>459</v>
       </c>
       <c r="D29" t="n">
-        <v>509.570375736621</v>
+        <v>633.570375736621</v>
       </c>
     </row>
   </sheetData>
@@ -25434,25 +25618,25 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>12</v>
+        <v>291</v>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E10" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F10" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G10" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -25463,10 +25647,10 @@
         <v>3</v>
       </c>
       <c r="C11" t="s">
-        <v>92</v>
+        <v>12</v>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11" t="s">
         <v>16</v>
@@ -25486,10 +25670,10 @@
         <v>3</v>
       </c>
       <c r="C12" t="s">
-        <v>127</v>
+        <v>92</v>
       </c>
       <c r="D12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E12" t="s">
         <v>16</v>
@@ -25509,10 +25693,10 @@
         <v>3</v>
       </c>
       <c r="C13" t="s">
-        <v>158</v>
+        <v>127</v>
       </c>
       <c r="D13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E13" t="s">
         <v>16</v>
@@ -25532,10 +25716,10 @@
         <v>3</v>
       </c>
       <c r="C14" t="s">
-        <v>176</v>
+        <v>158</v>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E14" t="s">
         <v>16</v>
@@ -25555,10 +25739,10 @@
         <v>3</v>
       </c>
       <c r="C15" t="s">
-        <v>203</v>
+        <v>176</v>
       </c>
       <c r="D15" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E15" t="s">
         <v>16</v>
@@ -25578,10 +25762,10 @@
         <v>3</v>
       </c>
       <c r="C16" t="s">
-        <v>237</v>
+        <v>203</v>
       </c>
       <c r="D16" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E16" t="s">
         <v>16</v>
@@ -25601,10 +25785,10 @@
         <v>3</v>
       </c>
       <c r="C17" t="s">
-        <v>262</v>
+        <v>237</v>
       </c>
       <c r="D17" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E17" t="s">
         <v>16</v>
@@ -25618,16 +25802,16 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C18" t="s">
-        <v>12</v>
+        <v>262</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E18" t="s">
         <v>16</v>
@@ -25641,16 +25825,16 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C19" t="s">
-        <v>92</v>
+        <v>291</v>
       </c>
       <c r="D19" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E19" t="s">
         <v>16</v>
@@ -25670,10 +25854,10 @@
         <v>4</v>
       </c>
       <c r="C20" t="s">
-        <v>127</v>
+        <v>12</v>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E20" t="s">
         <v>16</v>
@@ -25693,10 +25877,10 @@
         <v>4</v>
       </c>
       <c r="C21" t="s">
-        <v>158</v>
+        <v>92</v>
       </c>
       <c r="D21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E21" t="s">
         <v>16</v>
@@ -25716,10 +25900,10 @@
         <v>4</v>
       </c>
       <c r="C22" t="s">
-        <v>176</v>
+        <v>127</v>
       </c>
       <c r="D22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E22" t="s">
         <v>16</v>
@@ -25739,10 +25923,10 @@
         <v>4</v>
       </c>
       <c r="C23" t="s">
-        <v>203</v>
+        <v>158</v>
       </c>
       <c r="D23" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E23" t="s">
         <v>16</v>
@@ -25762,10 +25946,10 @@
         <v>4</v>
       </c>
       <c r="C24" t="s">
-        <v>237</v>
+        <v>176</v>
       </c>
       <c r="D24" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E24" t="s">
         <v>16</v>
@@ -25785,10 +25969,10 @@
         <v>4</v>
       </c>
       <c r="C25" t="s">
-        <v>262</v>
+        <v>203</v>
       </c>
       <c r="D25" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E25" t="s">
         <v>16</v>
@@ -25802,71 +25986,71 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C26" t="s">
-        <v>12</v>
+        <v>237</v>
       </c>
       <c r="D26" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E26" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F26" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G26" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C27" t="s">
-        <v>92</v>
+        <v>262</v>
       </c>
       <c r="D27" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E27" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F27" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G27" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B28" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C28" t="s">
-        <v>127</v>
+        <v>291</v>
       </c>
       <c r="D28" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E28" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F28" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G28" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="29">
@@ -25877,10 +26061,10 @@
         <v>5</v>
       </c>
       <c r="C29" t="s">
-        <v>158</v>
+        <v>12</v>
       </c>
       <c r="D29" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E29" t="s">
         <v>10</v>
@@ -25900,19 +26084,19 @@
         <v>5</v>
       </c>
       <c r="C30" t="s">
-        <v>176</v>
+        <v>92</v>
       </c>
       <c r="D30" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E30" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F30" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G30" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31">
@@ -25923,19 +26107,19 @@
         <v>5</v>
       </c>
       <c r="C31" t="s">
-        <v>203</v>
+        <v>127</v>
       </c>
       <c r="D31" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E31" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F31" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G31" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="32">
@@ -25946,10 +26130,10 @@
         <v>5</v>
       </c>
       <c r="C32" t="s">
-        <v>237</v>
+        <v>158</v>
       </c>
       <c r="D32" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E32" t="s">
         <v>10</v>
@@ -25969,10 +26153,10 @@
         <v>5</v>
       </c>
       <c r="C33" t="s">
-        <v>262</v>
+        <v>176</v>
       </c>
       <c r="D33" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E33" t="s">
         <v>16</v>
@@ -25986,39 +26170,39 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B34" t="n">
+        <v>5</v>
+      </c>
+      <c r="C34" t="s">
+        <v>203</v>
+      </c>
+      <c r="D34" t="n">
         <v>6</v>
       </c>
-      <c r="C34" t="s">
-        <v>12</v>
-      </c>
-      <c r="D34" t="n">
-        <v>1</v>
-      </c>
       <c r="E34" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F34" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G34" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B35" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C35" t="s">
-        <v>92</v>
+        <v>237</v>
       </c>
       <c r="D35" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E35" t="s">
         <v>10</v>
@@ -26032,39 +26216,39 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B36" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C36" t="s">
-        <v>127</v>
+        <v>262</v>
       </c>
       <c r="D36" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E36" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F36" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G36" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B37" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C37" t="s">
-        <v>158</v>
+        <v>291</v>
       </c>
       <c r="D37" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E37" t="s">
         <v>10</v>
@@ -26084,10 +26268,10 @@
         <v>6</v>
       </c>
       <c r="C38" t="s">
-        <v>176</v>
+        <v>12</v>
       </c>
       <c r="D38" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E38" t="s">
         <v>10</v>
@@ -26107,10 +26291,10 @@
         <v>6</v>
       </c>
       <c r="C39" t="s">
-        <v>203</v>
+        <v>92</v>
       </c>
       <c r="D39" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E39" t="s">
         <v>10</v>
@@ -26130,10 +26314,10 @@
         <v>6</v>
       </c>
       <c r="C40" t="s">
-        <v>237</v>
+        <v>127</v>
       </c>
       <c r="D40" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E40" t="s">
         <v>10</v>
@@ -26153,10 +26337,10 @@
         <v>6</v>
       </c>
       <c r="C41" t="s">
-        <v>262</v>
+        <v>158</v>
       </c>
       <c r="D41" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E41" t="s">
         <v>10</v>
@@ -26170,16 +26354,16 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="B42" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C42" t="s">
-        <v>12</v>
+        <v>176</v>
       </c>
       <c r="D42" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E42" t="s">
         <v>10</v>
@@ -26193,94 +26377,94 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="B43" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C43" t="s">
-        <v>92</v>
+        <v>203</v>
       </c>
       <c r="D43" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E43" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F43" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G43" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="B44" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C44" t="s">
-        <v>127</v>
+        <v>237</v>
       </c>
       <c r="D44" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E44" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F44" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G44" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="B45" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C45" t="s">
-        <v>158</v>
+        <v>262</v>
       </c>
       <c r="D45" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E45" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F45" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G45" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="B46" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C46" t="s">
-        <v>176</v>
+        <v>291</v>
       </c>
       <c r="D46" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E46" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F46" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G46" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="47">
@@ -26291,19 +26475,19 @@
         <v>2</v>
       </c>
       <c r="C47" t="s">
-        <v>203</v>
+        <v>12</v>
       </c>
       <c r="D47" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E47" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F47" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G47" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="48">
@@ -26314,10 +26498,10 @@
         <v>2</v>
       </c>
       <c r="C48" t="s">
-        <v>237</v>
+        <v>92</v>
       </c>
       <c r="D48" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E48" t="s">
         <v>16</v>
@@ -26337,10 +26521,10 @@
         <v>2</v>
       </c>
       <c r="C49" t="s">
-        <v>262</v>
+        <v>127</v>
       </c>
       <c r="D49" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E49" t="s">
         <v>16</v>
@@ -26354,140 +26538,140 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="B50" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C50" t="s">
-        <v>12</v>
+        <v>158</v>
       </c>
       <c r="D50" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E50" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F50" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G50" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="B51" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C51" t="s">
-        <v>92</v>
+        <v>176</v>
       </c>
       <c r="D51" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E51" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F51" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G51" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="B52" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C52" t="s">
-        <v>127</v>
+        <v>203</v>
       </c>
       <c r="D52" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E52" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F52" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G52" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="B53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" t="s">
+        <v>237</v>
+      </c>
+      <c r="D53" t="n">
         <v>7</v>
       </c>
-      <c r="C53" t="s">
-        <v>158</v>
-      </c>
-      <c r="D53" t="n">
-        <v>4</v>
-      </c>
       <c r="E53" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F53" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G53" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="B54" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C54" t="s">
-        <v>176</v>
+        <v>262</v>
       </c>
       <c r="D54" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E54" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F54" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G54" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="B55" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C55" t="s">
-        <v>203</v>
+        <v>291</v>
       </c>
       <c r="D55" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E55" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F55" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G55" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="56">
@@ -26498,10 +26682,10 @@
         <v>7</v>
       </c>
       <c r="C56" t="s">
-        <v>237</v>
+        <v>12</v>
       </c>
       <c r="D56" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E56" t="s">
         <v>10</v>
@@ -26521,10 +26705,10 @@
         <v>7</v>
       </c>
       <c r="C57" t="s">
-        <v>262</v>
+        <v>92</v>
       </c>
       <c r="D57" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E57" t="s">
         <v>10</v>
@@ -26538,16 +26722,16 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="B58" t="n">
-        <v>8.2</v>
+        <v>7</v>
       </c>
       <c r="C58" t="s">
-        <v>12</v>
+        <v>127</v>
       </c>
       <c r="D58" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E58" t="s">
         <v>10</v>
@@ -26561,16 +26745,16 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="B59" t="n">
-        <v>8.2</v>
+        <v>7</v>
       </c>
       <c r="C59" t="s">
-        <v>92</v>
+        <v>158</v>
       </c>
       <c r="D59" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E59" t="s">
         <v>10</v>
@@ -26584,16 +26768,16 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="B60" t="n">
-        <v>8.2</v>
+        <v>7</v>
       </c>
       <c r="C60" t="s">
-        <v>127</v>
+        <v>176</v>
       </c>
       <c r="D60" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E60" t="s">
         <v>10</v>
@@ -26607,16 +26791,16 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="B61" t="n">
-        <v>8.2</v>
+        <v>7</v>
       </c>
       <c r="C61" t="s">
-        <v>158</v>
+        <v>203</v>
       </c>
       <c r="D61" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E61" t="s">
         <v>10</v>
@@ -26630,16 +26814,16 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="B62" t="n">
-        <v>8.2</v>
+        <v>7</v>
       </c>
       <c r="C62" t="s">
-        <v>176</v>
+        <v>237</v>
       </c>
       <c r="D62" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E62" t="s">
         <v>10</v>
@@ -26653,16 +26837,16 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="B63" t="n">
-        <v>8.2</v>
+        <v>7</v>
       </c>
       <c r="C63" t="s">
-        <v>203</v>
+        <v>262</v>
       </c>
       <c r="D63" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E63" t="s">
         <v>10</v>
@@ -26676,16 +26860,16 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="B64" t="n">
-        <v>8.2</v>
+        <v>7</v>
       </c>
       <c r="C64" t="s">
-        <v>237</v>
+        <v>291</v>
       </c>
       <c r="D64" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E64" t="s">
         <v>10</v>
@@ -26705,10 +26889,10 @@
         <v>8.2</v>
       </c>
       <c r="C65" t="s">
-        <v>262</v>
+        <v>12</v>
       </c>
       <c r="D65" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E65" t="s">
         <v>10</v>
@@ -26717,6 +26901,190 @@
         <v>11</v>
       </c>
       <c r="G65" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s">
+        <v>467</v>
+      </c>
+      <c r="B66" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>92</v>
+      </c>
+      <c r="D66" t="n">
+        <v>2</v>
+      </c>
+      <c r="E66" t="s">
+        <v>10</v>
+      </c>
+      <c r="F66" t="s">
+        <v>11</v>
+      </c>
+      <c r="G66" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s">
+        <v>467</v>
+      </c>
+      <c r="B67" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C67" t="s">
+        <v>127</v>
+      </c>
+      <c r="D67" t="n">
+        <v>3</v>
+      </c>
+      <c r="E67" t="s">
+        <v>10</v>
+      </c>
+      <c r="F67" t="s">
+        <v>11</v>
+      </c>
+      <c r="G67" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s">
+        <v>467</v>
+      </c>
+      <c r="B68" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>158</v>
+      </c>
+      <c r="D68" t="n">
+        <v>4</v>
+      </c>
+      <c r="E68" t="s">
+        <v>10</v>
+      </c>
+      <c r="F68" t="s">
+        <v>11</v>
+      </c>
+      <c r="G68" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s">
+        <v>467</v>
+      </c>
+      <c r="B69" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C69" t="s">
+        <v>176</v>
+      </c>
+      <c r="D69" t="n">
+        <v>5</v>
+      </c>
+      <c r="E69" t="s">
+        <v>10</v>
+      </c>
+      <c r="F69" t="s">
+        <v>11</v>
+      </c>
+      <c r="G69" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s">
+        <v>467</v>
+      </c>
+      <c r="B70" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>203</v>
+      </c>
+      <c r="D70" t="n">
+        <v>6</v>
+      </c>
+      <c r="E70" t="s">
+        <v>10</v>
+      </c>
+      <c r="F70" t="s">
+        <v>11</v>
+      </c>
+      <c r="G70" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="s">
+        <v>467</v>
+      </c>
+      <c r="B71" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C71" t="s">
+        <v>237</v>
+      </c>
+      <c r="D71" t="n">
+        <v>7</v>
+      </c>
+      <c r="E71" t="s">
+        <v>10</v>
+      </c>
+      <c r="F71" t="s">
+        <v>11</v>
+      </c>
+      <c r="G71" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s">
+        <v>467</v>
+      </c>
+      <c r="B72" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C72" t="s">
+        <v>262</v>
+      </c>
+      <c r="D72" t="n">
+        <v>8</v>
+      </c>
+      <c r="E72" t="s">
+        <v>10</v>
+      </c>
+      <c r="F72" t="s">
+        <v>11</v>
+      </c>
+      <c r="G72" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s">
+        <v>467</v>
+      </c>
+      <c r="B73" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="C73" t="s">
+        <v>291</v>
+      </c>
+      <c r="D73" t="n">
+        <v>9</v>
+      </c>
+      <c r="E73" t="s">
+        <v>10</v>
+      </c>
+      <c r="F73" t="s">
+        <v>11</v>
+      </c>
+      <c r="G73" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>